<commit_message>
Update feature extraction method documentation and remove obsolete files
</commit_message>
<xml_diff>
--- a/Mambapro实验.xlsx
+++ b/Mambapro实验.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23720" windowHeight="11520"/>
+    <workbookView windowWidth="25600" windowHeight="10600"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
     <t>/</t>
   </si>
   <si>
-    <t>三尺度&amp;MLP简单拼接&amp;专家网络</t>
+    <t>三尺度&amp;MLP简单拼接&amp;专家网络MoE</t>
   </si>
   <si>
     <t xml:space="preserve">./run_experiment.sh   --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml   </t>
@@ -208,6 +208,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -244,6 +251,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -280,6 +294,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -313,6 +334,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -349,6 +377,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -382,6 +417,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -418,6 +460,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -451,6 +500,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -489,6 +545,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -522,6 +585,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>cd /home/zubuntu/workspace/yzy/MambaPro
 bash run_experiment.sh \
     --config_file configs/RGBNT201/</t>
@@ -611,6 +681,14 @@
   </numFmts>
   <fonts count="23">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
@@ -776,33 +854,13 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="40">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1162,64 +1220,70 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1228,10 +1292,10 @@
     <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1240,10 +1304,10 @@
     <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1252,10 +1316,10 @@
     <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1264,10 +1328,10 @@
     <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1276,26 +1340,23 @@
     <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1303,12 +1364,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1317,7 +1372,19 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1326,7 +1393,34 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1341,22 +1435,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1664,8 +1743,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7447915" y="14472285"/>
-          <a:ext cx="2463800" cy="558800"/>
+          <a:off x="8178800" y="12217400"/>
+          <a:ext cx="2463800" cy="347345"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1702,7 +1781,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7265670" y="19492595"/>
+          <a:off x="7996555" y="16127095"/>
           <a:ext cx="2500630" cy="554355"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1740,7 +1819,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7473950" y="13124180"/>
+          <a:off x="8204835" y="11013440"/>
           <a:ext cx="2475230" cy="544830"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1778,7 +1857,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7266305" y="16807815"/>
+          <a:off x="7997190" y="14049375"/>
           <a:ext cx="2528570" cy="542290"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1816,7 +1895,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7265035" y="36259135"/>
+          <a:off x="7995920" y="30914975"/>
           <a:ext cx="2837815" cy="732790"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1854,7 +1933,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7286625" y="41793795"/>
+          <a:off x="8017510" y="36055935"/>
           <a:ext cx="2899410" cy="770890"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1892,7 +1971,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7287260" y="46816645"/>
+          <a:off x="8018145" y="41078785"/>
           <a:ext cx="2903855" cy="689610"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1912,8 +1991,8 @@
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>2787650</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>1781810</xdr:rowOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>3810</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1930,7 +2009,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16334105" y="12875260"/>
+          <a:off x="17578705" y="10764520"/>
           <a:ext cx="2615565" cy="1456690"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2194,878 +2273,787 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:S27"/>
-  <sheetFormatPr defaultColWidth="9.02884615384615" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="9.02727272727273" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="33.6442307692308" style="1" customWidth="1"/>
-    <col min="2" max="2" width="76.2019230769231" style="2" customWidth="1"/>
-    <col min="3" max="3" width="44.7980769230769" style="3" customWidth="1"/>
-    <col min="4" max="7" width="9.02884615384615" style="1"/>
-    <col min="8" max="8" width="53.9711538461538" style="4" customWidth="1"/>
-    <col min="9" max="9" width="49.5961538461538" style="5" customWidth="1"/>
-    <col min="10" max="13" width="9.02884615384615" style="1"/>
-    <col min="14" max="14" width="80.6442307692308" style="4" customWidth="1"/>
-    <col min="15" max="15" width="35.9807692307692" style="5" customWidth="1"/>
-    <col min="16" max="16384" width="9.02884615384615" style="1"/>
+    <col min="1" max="1" width="38.1181818181818" style="2" customWidth="1"/>
+    <col min="2" max="2" width="76.2" style="3" customWidth="1"/>
+    <col min="3" max="3" width="44.8" style="4" customWidth="1"/>
+    <col min="4" max="7" width="9.02727272727273" style="2"/>
+    <col min="8" max="8" width="53.9727272727273" style="3" customWidth="1"/>
+    <col min="9" max="9" width="49.6" style="4" customWidth="1"/>
+    <col min="10" max="13" width="9.02727272727273" style="2"/>
+    <col min="14" max="14" width="80.6454545454545" style="3" customWidth="1"/>
+    <col min="15" max="15" width="35.9818181818182" style="4" customWidth="1"/>
+    <col min="16" max="16384" width="9.02727272727273" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19">
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="1:19">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="D1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="6" t="s">
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18" t="s">
+      <c r="J1" s="8"/>
+      <c r="K1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="6" t="s">
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="P1" s="20" t="s">
+      <c r="P1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
     </row>
-    <row r="2" spans="4:19">
-      <c r="D2" s="9" t="s">
+    <row r="2" spans="1:19">
+      <c r="D2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="19" t="s">
+      <c r="J2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="K2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="19" t="s">
+      <c r="L2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="19" t="s">
+      <c r="M2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="2"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="Q2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="S2" s="21" t="s">
+      <c r="S2" s="12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
-      <c r="A3" s="1" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:19">
+      <c r="A3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="9">
+      <c r="B3" s="14"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="16">
         <v>78.9</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="16">
         <v>83.4</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="16">
         <v>89.8</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="16">
         <v>91.9</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="19">
+      <c r="H3" s="14"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="17">
         <v>83.9</v>
       </c>
-      <c r="K3" s="19">
+      <c r="K3" s="17">
         <v>94.7</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="21">
+      <c r="N3" s="14"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="19">
         <v>56.5</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="Q3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="R3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="S3" s="21">
+      <c r="S3" s="19">
         <v>47</v>
       </c>
     </row>
     <row r="4" ht="248" customHeight="1" spans="1:19">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="23">
         <v>80.7</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="23">
         <v>85.2</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="23">
         <v>91.1</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="23">
         <v>94</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="19">
+      <c r="J4" s="11">
         <v>79.2</v>
       </c>
-      <c r="K4" s="19">
+      <c r="K4" s="11">
         <v>93.3</v>
       </c>
-      <c r="L4" s="19">
+      <c r="L4" s="11">
         <v>94.2</v>
       </c>
-      <c r="M4" s="19">
+      <c r="M4" s="11">
         <v>95</v>
       </c>
-      <c r="N4" s="16" t="s">
+      <c r="N4" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="O4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
-      <c r="S4" s="21"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
     </row>
-    <row r="5" spans="2:19">
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="9">
+    <row r="5" spans="1:19">
+      <c r="B5" s="24"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="23">
         <v>80.2</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="23">
         <v>83.9</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="23">
         <v>89.4</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="23">
         <v>92.3</v>
       </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="19">
+      <c r="H5" s="24"/>
+      <c r="J5" s="11">
         <v>79.8</v>
       </c>
-      <c r="K5" s="19">
+      <c r="K5" s="11">
         <v>94.2</v>
       </c>
-      <c r="L5" s="19">
+      <c r="L5" s="11">
         <v>95.3</v>
       </c>
-      <c r="M5" s="19">
+      <c r="M5" s="11">
         <v>95.6</v>
       </c>
-      <c r="N5" s="2"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
     </row>
-    <row r="6" ht="320" spans="2:19">
-      <c r="B6" s="12"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="9">
+    <row r="6" ht="224" spans="1:19">
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="23">
         <v>80.3</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="23">
         <v>84.7</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="23">
         <v>91.9</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="23">
         <v>94.6</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="19">
+      <c r="J6" s="11">
         <v>80.4</v>
       </c>
-      <c r="K6" s="19">
+      <c r="K6" s="11">
         <v>92.7</v>
       </c>
-      <c r="L6" s="19">
+      <c r="L6" s="11">
         <v>94.2</v>
       </c>
-      <c r="M6" s="19">
+      <c r="M6" s="11">
         <v>95</v>
       </c>
-      <c r="N6" s="2"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
     </row>
-    <row r="7" ht="353" spans="2:19">
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="12" t="s">
+    <row r="7" ht="294" spans="1:19">
+      <c r="B7" s="24"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="12"/>
     </row>
-    <row r="8" ht="168" spans="1:19">
-      <c r="A8" s="1" t="s">
+    <row r="8" ht="140" spans="1:19">
+      <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="9">
+      <c r="C8" s="25"/>
+      <c r="D8" s="10">
         <v>78.5</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="10">
         <v>82.4</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="10">
         <v>88.5</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="10">
         <v>90.9</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="19">
+      <c r="J8" s="11">
         <v>80.7</v>
       </c>
-      <c r="K8" s="19">
+      <c r="K8" s="11">
         <v>94.2</v>
       </c>
-      <c r="L8" s="19">
+      <c r="L8" s="11">
         <v>95.4</v>
       </c>
-      <c r="M8" s="19">
+      <c r="M8" s="11">
         <v>96.2</v>
       </c>
-      <c r="N8" s="2"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
     </row>
-    <row r="9" ht="135" spans="2:19">
-      <c r="B9" s="14" t="s">
+    <row r="9" ht="112" spans="1:19">
+      <c r="B9" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="10">
         <v>73.4</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="10">
         <v>76.2</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="10">
         <v>84.9</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="10">
         <v>89.7</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
-      <c r="R9" s="21"/>
-      <c r="S9" s="21"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
     </row>
-    <row r="10" ht="185" spans="2:19">
-      <c r="B10" s="14" t="s">
+    <row r="10" ht="140" spans="1:19">
+      <c r="B10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="10">
         <v>74.6</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="10">
         <v>77.2</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="10">
         <v>86</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="10">
         <v>89.2</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
-      <c r="S10" s="21"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="21"/>
-      <c r="S11" s="21"/>
+      <c r="B11" s="24"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
     </row>
-    <row r="12" ht="135" spans="2:19">
-      <c r="B12" s="12" t="s">
+    <row r="12" ht="112" spans="1:19">
+      <c r="B12" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="9">
+      <c r="C12" s="25"/>
+      <c r="D12" s="10">
         <v>76.9</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="10">
         <v>79.9</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="10">
         <v>88.5</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="10">
         <v>92.2</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="21"/>
-      <c r="Q12" s="21"/>
-      <c r="R12" s="21"/>
-      <c r="S12" s="21"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
     </row>
-    <row r="13" spans="4:19">
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="21"/>
-      <c r="Q13" s="21"/>
-      <c r="R13" s="21"/>
-      <c r="S13" s="21"/>
+    <row r="13" spans="1:19">
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
     </row>
     <row r="14" ht="240" customHeight="1" spans="1:19">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="10">
         <v>77.5</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="10">
         <v>82.9</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="10">
         <v>90.8</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="10">
         <v>93.2</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="21"/>
-      <c r="Q14" s="21"/>
-      <c r="R14" s="21"/>
-      <c r="S14" s="21"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
     </row>
-    <row r="15" ht="152" spans="2:19">
-      <c r="B15" s="14" t="s">
+    <row r="15" ht="126" spans="1:19">
+      <c r="B15" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="10">
         <v>73.9</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="10">
         <v>75.2</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="10">
         <v>83.9</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="10">
         <v>88</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="21"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="21"/>
-      <c r="S15" s="21"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
     </row>
-    <row r="16" ht="152" spans="1:19">
-      <c r="A16" s="1" t="s">
+    <row r="16" ht="126" spans="1:19">
+      <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="10">
         <v>77</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="10">
         <v>77.6</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="10">
         <v>87</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="10">
         <v>90.1</v>
       </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="21"/>
-      <c r="S16" s="21"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="12"/>
     </row>
-    <row r="17" ht="152" spans="2:19">
-      <c r="B17" s="14" t="s">
+    <row r="17" ht="126" spans="1:19">
+      <c r="B17" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="10">
         <v>76.3</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="10">
         <v>79.7</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="10">
         <v>89.6</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="10">
         <v>92.5</v>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="21"/>
-      <c r="Q17" s="21"/>
-      <c r="R17" s="21"/>
-      <c r="S17" s="21"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="12"/>
     </row>
-    <row r="18" ht="152" spans="1:19">
-      <c r="A18" s="1" t="s">
+    <row r="18" ht="126" spans="1:19">
+      <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="21"/>
-      <c r="Q18" s="21"/>
-      <c r="R18" s="21"/>
-      <c r="S18" s="21"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
     </row>
-    <row r="19" ht="152" spans="2:19">
-      <c r="B19" s="14" t="s">
+    <row r="19" ht="126" spans="1:19">
+      <c r="B19" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <v>74.4</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="10">
         <v>76.8</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="10">
         <v>87.3</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="10">
         <v>90.8</v>
       </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="21"/>
-      <c r="Q19" s="21"/>
-      <c r="R19" s="21"/>
-      <c r="S19" s="21"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
+      <c r="S19" s="12"/>
     </row>
     <row r="20" ht="196" customHeight="1" spans="1:19">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <v>75.2</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="10">
         <v>78.8</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="10">
         <v>87.9</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="10">
         <v>91.9</v>
       </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="21"/>
-      <c r="Q20" s="21"/>
-      <c r="R20" s="21"/>
-      <c r="S20" s="21"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
+      <c r="P20" s="12"/>
+      <c r="Q20" s="12"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="12"/>
     </row>
-    <row r="21" ht="185" spans="2:19">
-      <c r="B21" s="14" t="s">
+    <row r="21" ht="154" spans="1:19">
+      <c r="B21" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="10">
         <v>73</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="10">
         <v>73.9</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="10">
         <v>84.7</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="10">
         <v>88.4</v>
       </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="3"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="S21" s="21"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
     </row>
     <row r="22" ht="197" customHeight="1" spans="1:19">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="10">
         <v>70.9</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="10">
         <v>73.4</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="10">
         <v>81.6</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="10">
         <v>87.9</v>
       </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="21"/>
-      <c r="Q22" s="21"/>
-      <c r="R22" s="21"/>
-      <c r="S22" s="21"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="11"/>
+      <c r="P22" s="12"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="12"/>
     </row>
-    <row r="23" ht="208" customHeight="1" spans="2:19">
-      <c r="B23" s="14" t="s">
+    <row r="23" ht="208" customHeight="1" spans="1:19">
+      <c r="B23" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="10">
         <v>75.9</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="10">
         <v>77</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="10">
         <v>85.6</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="10">
         <v>89.8</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="3"/>
-      <c r="P23" s="21"/>
-      <c r="Q23" s="21"/>
-      <c r="R23" s="21"/>
-      <c r="S23" s="21"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
     </row>
     <row r="24" ht="179" customHeight="1" spans="1:19">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="21"/>
-      <c r="Q24" s="21"/>
-      <c r="R24" s="21"/>
-      <c r="S24" s="21"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
     </row>
-    <row r="25" ht="217" customHeight="1" spans="2:19">
-      <c r="B25" s="16" t="s">
+    <row r="25" ht="217" customHeight="1" spans="1:19">
+      <c r="B25" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="10">
         <v>75.8</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="10">
         <v>81.7</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="10">
         <v>89</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="10">
         <v>92.6</v>
       </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="3"/>
-      <c r="P25" s="21"/>
-      <c r="Q25" s="21"/>
-      <c r="R25" s="21"/>
-      <c r="S25" s="21"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+      <c r="M25" s="11"/>
+      <c r="P25" s="12"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="12"/>
     </row>
     <row r="26" ht="180" customHeight="1" spans="1:19">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B26" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="10">
         <v>78.9</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="10">
         <v>82.5</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F26" s="10">
         <v>90.2</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="10">
         <v>92.7</v>
       </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="3"/>
-      <c r="P26" s="21"/>
-      <c r="Q26" s="21"/>
-      <c r="R26" s="21"/>
-      <c r="S26" s="21"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="11"/>
+      <c r="M26" s="11"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="12"/>
     </row>
     <row r="27" spans="1:19">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="19"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="3"/>
-      <c r="P27" s="21"/>
-      <c r="Q27" s="21"/>
-      <c r="R27" s="21"/>
-      <c r="S27" s="21"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="11"/>
+      <c r="M27" s="11"/>
+      <c r="P27" s="12"/>
+      <c r="Q27" s="12"/>
+      <c r="R27" s="12"/>
+      <c r="S27" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Update model loading to read pre-trained path from config and ensure UTF-8 encoding for log files
</commit_message>
<xml_diff>
--- a/Mambapro实验.xlsx
+++ b/Mambapro实验.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="10600"/>
+    <workbookView windowWidth="11930" windowHeight="6600"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1350,7 +1350,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1390,9 +1390,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1403,12 +1400,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
@@ -1743,7 +1734,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8178800" y="12217400"/>
+          <a:off x="9195435" y="12217400"/>
           <a:ext cx="2463800" cy="347345"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1781,7 +1772,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7996555" y="16127095"/>
+          <a:off x="9013190" y="16127095"/>
           <a:ext cx="2500630" cy="554355"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1819,7 +1810,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8204835" y="11013440"/>
+          <a:off x="9221470" y="11013440"/>
           <a:ext cx="2475230" cy="544830"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1857,7 +1848,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7997190" y="14049375"/>
+          <a:off x="9013825" y="14049375"/>
           <a:ext cx="2528570" cy="542290"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1895,7 +1886,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7995920" y="30914975"/>
+          <a:off x="9012555" y="30914975"/>
           <a:ext cx="2837815" cy="732790"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1933,7 +1924,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8017510" y="36055935"/>
+          <a:off x="9034145" y="36055935"/>
           <a:ext cx="2899410" cy="770890"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1971,7 +1962,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8018145" y="41078785"/>
+          <a:off x="9034780" y="41078785"/>
           <a:ext cx="2903855" cy="689610"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2009,7 +2000,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17578705" y="10764520"/>
+          <a:off x="18595340" y="10764520"/>
           <a:ext cx="2615565" cy="1456690"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2276,7 +2267,7 @@
   <sheetFormatPr defaultColWidth="9.02727272727273" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="38.1181818181818" style="2" customWidth="1"/>
-    <col min="2" max="2" width="76.2" style="3" customWidth="1"/>
+    <col min="2" max="2" width="90.7545454545455" style="3" customWidth="1"/>
     <col min="3" max="3" width="44.8" style="4" customWidth="1"/>
     <col min="4" max="7" width="9.02727272727273" style="2"/>
     <col min="8" max="8" width="53.9727272727273" style="3" customWidth="1"/>
@@ -2364,72 +2355,72 @@
       </c>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:19">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16">
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15">
         <v>78.9</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="15">
         <v>83.4</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="15">
         <v>89.8</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="15">
         <v>91.9</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="17">
+      <c r="H3" s="13"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="16">
         <v>83.9</v>
       </c>
-      <c r="K3" s="17">
+      <c r="K3" s="16">
         <v>94.7</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="14"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="19">
+      <c r="N3" s="13"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="17">
         <v>56.5</v>
       </c>
-      <c r="Q3" s="20" t="s">
+      <c r="Q3" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="R3" s="20" t="s">
+      <c r="R3" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="S3" s="19">
+      <c r="S3" s="17">
         <v>47</v>
       </c>
     </row>
     <row r="4" ht="248" customHeight="1" spans="1:19">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="20">
         <v>80.7</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="20">
         <v>85.2</v>
       </c>
-      <c r="F4" s="23">
+      <c r="F4" s="20">
         <v>91.1</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="20">
         <v>94</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="21" t="s">
         <v>13</v>
       </c>
       <c r="J4" s="11">
@@ -2444,7 +2435,7 @@
       <c r="M4" s="11">
         <v>95</v>
       </c>
-      <c r="N4" s="24" t="s">
+      <c r="N4" s="21" t="s">
         <v>14</v>
       </c>
       <c r="O4" s="4" t="s">
@@ -2456,21 +2447,21 @@
       <c r="S4" s="12"/>
     </row>
     <row r="5" spans="1:19">
-      <c r="B5" s="24"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="23">
+      <c r="B5" s="21"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="20">
         <v>80.2</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="20">
         <v>83.9</v>
       </c>
-      <c r="F5" s="23">
+      <c r="F5" s="20">
         <v>89.4</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="20">
         <v>92.3</v>
       </c>
-      <c r="H5" s="24"/>
+      <c r="H5" s="21"/>
       <c r="J5" s="11">
         <v>79.8</v>
       </c>
@@ -2489,21 +2480,21 @@
       <c r="S5" s="12"/>
     </row>
     <row r="6" ht="224" spans="1:19">
-      <c r="B6" s="24"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="23">
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="20">
         <v>80.3</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="20">
         <v>84.7</v>
       </c>
-      <c r="F6" s="23">
+      <c r="F6" s="20">
         <v>91.9</v>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="20">
         <v>94.6</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="21" t="s">
         <v>13</v>
       </c>
       <c r="J6" s="11">
@@ -2524,13 +2515,13 @@
       <c r="S6" s="12"/>
     </row>
     <row r="7" ht="294" spans="1:19">
-      <c r="B7" s="24"/>
-      <c r="C7" s="25"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="21" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="11"/>
@@ -2546,10 +2537,10 @@
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="25"/>
+      <c r="C8" s="22"/>
       <c r="D8" s="10">
         <v>78.5</v>
       </c>
@@ -2562,7 +2553,7 @@
       <c r="G8" s="10">
         <v>90.9</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="21" t="s">
         <v>19</v>
       </c>
       <c r="J8" s="11">
@@ -2583,7 +2574,7 @@
       <c r="S8" s="12"/>
     </row>
     <row r="9" ht="112" spans="1:19">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="23" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="10">
@@ -2608,7 +2599,7 @@
       <c r="S9" s="12"/>
     </row>
     <row r="10" ht="140" spans="1:19">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="23" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="10">
@@ -2636,7 +2627,7 @@
       <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="24"/>
+      <c r="B11" s="21"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -2651,10 +2642,10 @@
       <c r="S11" s="12"/>
     </row>
     <row r="12" ht="112" spans="1:19">
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="25"/>
+      <c r="C12" s="22"/>
       <c r="D12" s="10">
         <v>76.9</v>
       </c>
@@ -2694,10 +2685,10 @@
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="24" t="s">
         <v>26</v>
       </c>
       <c r="D14" s="10">
@@ -2722,7 +2713,7 @@
       <c r="S14" s="12"/>
     </row>
     <row r="15" ht="126" spans="1:19">
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="23" t="s">
         <v>27</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -2753,7 +2744,7 @@
       <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="23" t="s">
         <v>29</v>
       </c>
       <c r="C16" s="4" t="s">
@@ -2781,7 +2772,7 @@
       <c r="S16" s="12"/>
     </row>
     <row r="17" ht="126" spans="1:19">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="23" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="4" t="s">
@@ -2812,7 +2803,7 @@
       <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="4" t="s">
@@ -2832,7 +2823,7 @@
       <c r="S18" s="12"/>
     </row>
     <row r="19" ht="126" spans="1:19">
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="23" t="s">
         <v>33</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -2863,7 +2854,7 @@
       <c r="A20" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="23" t="s">
         <v>35</v>
       </c>
       <c r="D20" s="10">
@@ -2888,7 +2879,7 @@
       <c r="S20" s="12"/>
     </row>
     <row r="21" ht="154" spans="1:19">
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="23" t="s">
         <v>36</v>
       </c>
       <c r="D21" s="10">
@@ -2916,7 +2907,7 @@
       <c r="A22" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="23" t="s">
         <v>38</v>
       </c>
       <c r="D22" s="10">
@@ -2941,7 +2932,7 @@
       <c r="S22" s="12"/>
     </row>
     <row r="23" ht="208" customHeight="1" spans="1:19">
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="23" t="s">
         <v>39</v>
       </c>
       <c r="D23" s="10">
@@ -2969,7 +2960,7 @@
       <c r="A24" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="21" t="s">
         <v>41</v>
       </c>
       <c r="D24" s="10"/>
@@ -2986,7 +2977,7 @@
       <c r="S24" s="12"/>
     </row>
     <row r="25" ht="217" customHeight="1" spans="1:19">
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="21" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="10">
@@ -3014,7 +3005,7 @@
       <c r="A26" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="21" t="s">
         <v>44</v>
       </c>
       <c r="D26" s="10">
@@ -3039,7 +3030,7 @@
       <c r="S26" s="12"/>
     </row>
     <row r="27" spans="1:19">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="25" t="s">
         <v>45</v>
       </c>
       <c r="D27" s="10"/>

</xml_diff>

<commit_message>
Refine MambaPro configuration parameters for MoE optimization, enhancing expert network performance and adjusting loss weights for better task balance. Update documentation for clarity on new settings.
</commit_message>
<xml_diff>
--- a/Mambapro实验.xlsx
+++ b/Mambapro实验.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11930" windowHeight="6600"/>
+    <workbookView windowWidth="15780" windowHeight="10000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1772,7 +1772,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9013190" y="16127095"/>
+          <a:off x="9013190" y="15949295"/>
           <a:ext cx="2500630" cy="554355"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1886,7 +1886,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9012555" y="30914975"/>
+          <a:off x="9012555" y="30737175"/>
           <a:ext cx="2837815" cy="732790"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1924,7 +1924,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9034145" y="36055935"/>
+          <a:off x="9034145" y="35878135"/>
           <a:ext cx="2899410" cy="770890"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1962,7 +1962,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9034780" y="41078785"/>
+          <a:off x="9034780" y="40900985"/>
           <a:ext cx="2903855" cy="689610"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2598,7 +2598,7 @@
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
     </row>
-    <row r="10" ht="140" spans="1:19">
+    <row r="10" ht="126" spans="1:19">
       <c r="B10" s="23" t="s">
         <v>21</v>
       </c>

</xml_diff>